<commit_message>
feat(r3): complete requirement 3
</commit_message>
<xml_diff>
--- a/outputs/deliverables/reports/self_assessment.xlsx
+++ b/outputs/deliverables/reports/self_assessment.xlsx
@@ -455,7 +455,7 @@
         <v>25</v>
       </c>
       <c r="D4" t="str">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
@@ -512,7 +512,7 @@
         <v>100</v>
       </c>
       <c r="D8" t="str">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>